<commit_message>
Add Allure branding, EastWest logo, and theme customization
</commit_message>
<xml_diff>
--- a/testdata/EBAPI.xlsx
+++ b/testdata/EBAPI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARM83471\Playwright - API Automation Framework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0852864A-2617-4627-8376-3348D994B88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF73E5A-4D59-4FC1-83E1-81FE768B0106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="576" activeTab="3" xr2:uid="{E1A27D2B-6C2F-48BB-87D7-349C65AB89C7}"/>
   </bookViews>
@@ -42858,7 +42858,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -42935,7 +42935,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
@@ -42975,7 +42975,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
@@ -43015,7 +43015,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1" t="s">
@@ -43052,7 +43052,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1" t="s">
@@ -43089,7 +43089,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
@@ -43126,7 +43126,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
@@ -43163,7 +43163,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1" t="s">
@@ -43200,7 +43200,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="s">
@@ -43237,7 +43237,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
@@ -43274,7 +43274,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
@@ -43311,7 +43311,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1" t="s">
@@ -43348,7 +43348,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>915</v>
+        <v>17</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1" t="s">

</xml_diff>

<commit_message>
Code update for allure custom reports and write excel to max length to handle api response that exceeds
</commit_message>
<xml_diff>
--- a/testdata/EBAPI.xlsx
+++ b/testdata/EBAPI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARM83471\Playwright - API Automation Framework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF73E5A-4D59-4FC1-83E1-81FE768B0106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5185253-1C4F-4FAD-8C25-6A55495C1956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="576" activeTab="3" xr2:uid="{E1A27D2B-6C2F-48BB-87D7-349C65AB89C7}"/>
   </bookViews>
@@ -670,7 +670,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12622" uniqueCount="1847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12623" uniqueCount="1848">
   <si>
     <t>#</t>
   </si>
@@ -7192,6 +7192,9 @@
   </si>
   <si>
     <t>pLRFPZKifoRD00dj761QToHciekWqbbh</t>
+  </si>
+  <si>
+    <t>400,401,403</t>
   </si>
 </sst>
 </file>
@@ -7388,7 +7391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -7641,16 +7644,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="10" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -41588,31 +41588,31 @@
       <c r="H2" s="5">
         <v>200</v>
       </c>
-      <c r="I2" s="92" t="s">
+      <c r="I2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="92" t="s">
+      <c r="J2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="92" t="s">
+      <c r="L2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="93" t="s">
+      <c r="M2" s="6" t="s">
         <v>1839</v>
       </c>
-      <c r="N2" s="94" t="s">
+      <c r="N2" s="25" t="s">
         <v>1840</v>
       </c>
-      <c r="O2" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" s="95">
+      <c r="O2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q2" s="92" t="s">
+      <c r="Q2" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41642,31 +41642,30 @@
       <c r="H3" s="5">
         <v>400</v>
       </c>
-      <c r="I3" s="92" t="s">
+      <c r="I3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" s="92" t="s">
+      <c r="J3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="92" t="s">
+      <c r="L3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="93">
+      <c r="M3" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N3" s="94" t="s">
+      <c r="N3" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O3" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P3" s="95">
+      <c r="O3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P3" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q3" s="92"/>
     </row>
     <row r="4" spans="1:21" ht="60" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="str">
@@ -41691,29 +41690,29 @@
       <c r="H4" s="5">
         <v>400</v>
       </c>
-      <c r="I4" s="92" t="s">
+      <c r="I4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="92" t="s">
+      <c r="J4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="92" t="s">
+      <c r="L4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="93">
+      <c r="M4" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N4" s="94" t="s">
+      <c r="N4" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O4" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P4" s="95"/>
-      <c r="Q4" s="92" t="s">
+      <c r="O4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P4" s="92"/>
+      <c r="Q4" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41743,31 +41742,31 @@
       <c r="H5" s="88">
         <v>403</v>
       </c>
-      <c r="I5" s="92" t="s">
+      <c r="I5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="92" t="s">
+      <c r="J5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="92" t="s">
+      <c r="L5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="93">
+      <c r="M5" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N5" s="94" t="s">
+      <c r="N5" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O5" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P5" s="95">
+      <c r="O5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P5" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q5" s="92" t="s">
+      <c r="Q5" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41797,31 +41796,31 @@
       <c r="H6" s="5">
         <v>200</v>
       </c>
-      <c r="I6" s="92" t="s">
+      <c r="I6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="92" t="s">
+      <c r="J6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="92" t="s">
+      <c r="L6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="93" t="s">
+      <c r="M6" s="6" t="s">
         <v>1839</v>
       </c>
-      <c r="N6" s="94" t="s">
+      <c r="N6" s="25" t="s">
         <v>1840</v>
       </c>
-      <c r="O6" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P6" s="95">
+      <c r="O6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q6" s="92" t="s">
+      <c r="Q6" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41851,31 +41850,31 @@
       <c r="H7" s="4">
         <v>200</v>
       </c>
-      <c r="I7" s="92" t="s">
+      <c r="I7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J7" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K7" s="92" t="s">
+      <c r="J7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="92" t="s">
+      <c r="L7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M7" s="93">
+      <c r="M7" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N7" s="94" t="s">
+      <c r="N7" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O7" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P7" s="95">
+      <c r="O7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P7" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q7" s="92" t="s">
+      <c r="Q7" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41905,31 +41904,31 @@
       <c r="H8" s="4">
         <v>200</v>
       </c>
-      <c r="I8" s="92" t="s">
+      <c r="I8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K8" s="92" t="s">
+      <c r="J8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="92" t="s">
+      <c r="L8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="93" t="s">
+      <c r="M8" s="6" t="s">
         <v>1839</v>
       </c>
-      <c r="N8" s="94" t="s">
+      <c r="N8" s="25" t="s">
         <v>1840</v>
       </c>
-      <c r="O8" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P8" s="95">
+      <c r="O8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P8" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q8" s="92" t="s">
+      <c r="Q8" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -41959,31 +41958,31 @@
       <c r="H9" s="1">
         <v>401</v>
       </c>
-      <c r="I9" s="92" t="s">
+      <c r="I9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J9" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" s="92" t="s">
+      <c r="J9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L9" s="92" t="s">
+      <c r="L9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M9" s="93">
+      <c r="M9" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N9" s="94" t="s">
+      <c r="N9" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O9" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P9" s="95">
+      <c r="O9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P9" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q9" s="92" t="s">
+      <c r="Q9" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42013,31 +42012,31 @@
       <c r="H10" s="4">
         <v>200</v>
       </c>
-      <c r="I10" s="92" t="s">
+      <c r="I10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J10" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K10" s="92" t="s">
+      <c r="J10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L10" s="92" t="s">
+      <c r="L10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M10" s="93">
+      <c r="M10" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N10" s="94" t="s">
+      <c r="N10" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O10" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P10" s="95">
+      <c r="O10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P10" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q10" s="92" t="s">
+      <c r="Q10" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42067,31 +42066,31 @@
       <c r="H11" s="4">
         <v>400</v>
       </c>
-      <c r="I11" s="92" t="s">
+      <c r="I11" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J11" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K11" s="92" t="s">
+      <c r="J11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="92" t="s">
+      <c r="L11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="93">
+      <c r="M11" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N11" s="94" t="s">
+      <c r="N11" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O11" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P11" s="95">
+      <c r="O11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P11" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q11" s="92" t="s">
+      <c r="Q11" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42121,31 +42120,31 @@
       <c r="H12" s="4">
         <v>400</v>
       </c>
-      <c r="I12" s="92" t="s">
+      <c r="I12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J12" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K12" s="92" t="s">
+      <c r="J12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L12" s="92" t="s">
+      <c r="L12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="93">
+      <c r="M12" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N12" s="94" t="s">
+      <c r="N12" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O12" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P12" s="95">
+      <c r="O12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P12" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q12" s="92" t="s">
+      <c r="Q12" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42175,31 +42174,31 @@
       <c r="H13" s="4">
         <v>400</v>
       </c>
-      <c r="I13" s="92" t="s">
+      <c r="I13" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K13" s="92" t="s">
+      <c r="J13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L13" s="92" t="s">
+      <c r="L13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M13" s="93">
+      <c r="M13" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N13" s="94" t="s">
+      <c r="N13" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O13" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P13" s="95">
+      <c r="O13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P13" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q13" s="92" t="s">
+      <c r="Q13" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42229,31 +42228,31 @@
       <c r="H14" s="4">
         <v>400</v>
       </c>
-      <c r="I14" s="92" t="s">
+      <c r="I14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J14" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K14" s="92" t="s">
+      <c r="J14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L14" s="92" t="s">
+      <c r="L14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M14" s="93">
+      <c r="M14" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N14" s="94" t="s">
+      <c r="N14" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O14" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P14" s="95">
+      <c r="O14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P14" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q14" s="92" t="s">
+      <c r="Q14" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42283,31 +42282,31 @@
       <c r="H15" s="4">
         <v>200</v>
       </c>
-      <c r="I15" s="92" t="s">
+      <c r="I15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J15" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" s="92" t="s">
+      <c r="J15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L15" s="92" t="s">
+      <c r="L15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M15" s="93">
+      <c r="M15" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N15" s="94" t="s">
+      <c r="N15" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O15" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P15" s="95">
+      <c r="O15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P15" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q15" s="92" t="s">
+      <c r="Q15" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -42337,31 +42336,31 @@
       <c r="H16" s="4">
         <v>400</v>
       </c>
-      <c r="I16" s="92" t="s">
+      <c r="I16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J16" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="K16" s="92" t="s">
+      <c r="J16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L16" s="92" t="s">
+      <c r="L16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="M16" s="93">
+      <c r="M16" s="6">
         <v>1042346954</v>
       </c>
-      <c r="N16" s="94" t="s">
+      <c r="N16" s="25" t="s">
         <v>813</v>
       </c>
-      <c r="O16" s="92" t="s">
-        <v>23</v>
-      </c>
-      <c r="P16" s="95">
+      <c r="O16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="P16" s="92">
         <v>200061777902</v>
       </c>
-      <c r="Q16" s="92" t="s">
+      <c r="Q16" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -43326,7 +43325,7 @@
       <c r="G14" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="94">
         <v>200</v>
       </c>
       <c r="I14" s="1" t="str">
@@ -43363,8 +43362,8 @@
       <c r="G15" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="H15" s="16">
-        <v>400401403</v>
+      <c r="H15" s="93" t="s">
+        <v>1847</v>
       </c>
       <c r="I15" s="1" t="str">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Updates on VM for yaml
</commit_message>
<xml_diff>
--- a/testdata/EBAPI.xlsx
+++ b/testdata/EBAPI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARM83471\Playwright - API Automation Framework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55264320-A9A8-40AE-894F-5CFB7E931BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3C8C79-7F0D-4C7E-ADE6-01FDDC18DC06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Script Inventory" sheetId="1" r:id="rId1"/>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13435" uniqueCount="2377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13436" uniqueCount="2378">
   <si>
     <t>SandBox</t>
   </si>
@@ -8338,12 +8338,15 @@
   <si>
     <t>DuNZoeHA43ANE1CPKzAlXp8YVJPy0JmF</t>
   </si>
+  <si>
+    <t>For Execution</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8409,6 +8412,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -8600,7 +8611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="261">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9369,6 +9380,7 @@
     <xf numFmtId="49" fontId="2" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9733,28 +9745,32 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="B1:D22"/>
+  <dimension ref="B1:E22"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5703125" style="188" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.140625" style="188" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" style="195" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" style="196" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="188"/>
+    <col min="5" max="5" width="13.140625" style="188" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="188"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="189"/>
       <c r="D1" s="190"/>
     </row>
-    <row r="2" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="191" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="189"/>
       <c r="D2" s="190"/>
-    </row>
-    <row r="3" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E2" s="260" t="s">
+        <v>2377</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="192" t="s">
         <v>1</v>
       </c>
@@ -9762,8 +9778,12 @@
         <f>COUNTA(SBAuthAPI!E:E)-1</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E3" s="193">
+        <f>COUNTIF(SBAuthAPI!B:B,"Y")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C4" s="192" t="s">
         <v>2</v>
       </c>
@@ -9771,8 +9791,12 @@
         <f>COUNTA(SBBankList!E:E)-1</f>
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" s="193">
+        <f>COUNTIF(SBBankList!B:B,"Y")</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="192" t="s">
         <v>3</v>
       </c>
@@ -9780,8 +9804,12 @@
         <f>COUNTA(SBCheckStatus!E:E)-1</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="193">
+        <f>COUNTIF(SBCheckStatus!B:B,"Y")</f>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="192" t="s">
         <v>4</v>
       </c>
@@ -9789,22 +9817,30 @@
         <f>COUNTA(SBSendFunds!E:E)-1</f>
         <v>114</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E6" s="193">
+        <f>COUNTIF(SBSendFunds!B:B,"Y")</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C7" s="189"/>
       <c r="D7" s="194">
         <f>SUM(D3:D6)</f>
         <v>218</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E7" s="194">
+        <f>SUM(E3:E6)</f>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="191" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="189"/>
       <c r="D8" s="190"/>
     </row>
-    <row r="9" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="192" t="s">
         <v>1</v>
       </c>
@@ -9812,8 +9848,12 @@
         <f>COUNTA(PTTAuthAPI!E:E)-1</f>
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="193">
+        <f>COUNTIF(PTTAuthAPI!B:B,"Y")</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="192" t="s">
         <v>2</v>
       </c>
@@ -9821,8 +9861,12 @@
         <f>COUNTA(PTTBankList!E:E)-1</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="193">
+        <f>COUNTIF(PTTBankList!B:B,"Y")</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="192" t="s">
         <v>3</v>
       </c>
@@ -9830,8 +9874,12 @@
         <f>COUNTA(PTTCheckStatus!E:E)-1</f>
         <v>59</v>
       </c>
-    </row>
-    <row r="12" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="193">
+        <f>COUNTIF(PTTCheckStatus!B:B,"Y")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="192" t="s">
         <v>4</v>
       </c>
@@ -9839,22 +9887,30 @@
         <f>COUNTA(PTTSendFunds!E:E)-1</f>
         <v>230</v>
       </c>
-    </row>
-    <row r="13" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="193">
+        <f>COUNTIF(PTTSendFunds!B:B,"Y")</f>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C13" s="189"/>
       <c r="D13" s="194">
         <f>SUM(D9:D12)</f>
         <v>335</v>
       </c>
-    </row>
-    <row r="14" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E13" s="194">
+        <f>SUM(E9:E12)</f>
+        <v>211</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="191" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="189"/>
       <c r="D14" s="190"/>
     </row>
-    <row r="15" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="192" t="s">
         <v>1</v>
       </c>
@@ -9862,8 +9918,12 @@
         <f>COUNTA(PTLAuthAPI!E:E)-1</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="16" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E15" s="193">
+        <f>COUNTIF(PTLAuthAPI!B:B,"Y")</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="192" t="s">
         <v>2</v>
       </c>
@@ -9871,8 +9931,12 @@
         <f>COUNTA(PTLBankList!E:E)-1</f>
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="193">
+        <f>COUNTIF(PTLBankList!B:B,"Y")</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="192" t="s">
         <v>3</v>
       </c>
@@ -9880,8 +9944,12 @@
         <f>COUNTA(PTLCheckStatus!E:E)-1</f>
         <v>56</v>
       </c>
-    </row>
-    <row r="18" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="193">
+        <f>COUNTIF(PTLCheckStatus!B:B,"Y")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="192" t="s">
         <v>4</v>
       </c>
@@ -9889,29 +9957,41 @@
         <f>COUNTA(PTLSendFunds!E:E)-1</f>
         <v>190</v>
       </c>
-    </row>
-    <row r="19" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="193">
+        <f>COUNTIF(PTLSendFunds!B:B,"Y")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="189"/>
       <c r="D19" s="194">
         <f>SUM(D15:D18)</f>
         <v>291</v>
       </c>
-    </row>
-    <row r="20" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="194">
+        <f>SUM(E15:E18)</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="189"/>
       <c r="D20" s="190"/>
     </row>
-    <row r="21" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="189"/>
       <c r="D21" s="190"/>
     </row>
-    <row r="22" spans="3:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="191" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="194">
         <f>SUM(D7,D13,D19)</f>
         <v>844</v>
+      </c>
+      <c r="E22" s="194">
+        <f>SUM(E7,E13,E19)</f>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>